<commit_message>
codebase + docs backup 2026-06-27 00:20
</commit_message>
<xml_diff>
--- a/amc_book/SBI Mutual Fund/SBI Equity Hybrid Fund _G_/FACT_SHEET_2026-06-25.xlsx
+++ b/amc_book/SBI Mutual Fund/SBI Equity Hybrid Fund _G_/FACT_SHEET_2026-06-25.xlsx
@@ -618,34 +618,34 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>12125</v>
+        <v>73323</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>129550</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>157.0794</v>
+        <v>949.8995</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>129550</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>157.0794</v>
+        <v>949.8995</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>130120</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>157.7705</v>
+        <v>954.0789</v>
       </c>
       <c r="M6" s="9" t="n">
         <v>-0.4381</v>
       </c>
       <c r="N6" s="10" t="n">
-        <v>-0.00082</v>
+        <v>-0.00496</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.187</v>
+        <v>1.1311</v>
       </c>
     </row>
     <row r="7">
@@ -663,14 +663,14 @@
       <c r="H7" s="11" t="n"/>
       <c r="I7" s="11" t="n"/>
       <c r="J7" s="13" t="n">
-        <v>157.079</v>
+        <v>949.899</v>
       </c>
       <c r="K7" s="11" t="n"/>
       <c r="L7" s="11" t="n"/>
       <c r="M7" s="11" t="n"/>
       <c r="N7" s="11" t="n"/>
       <c r="O7" s="14" t="n">
-        <v>0.19</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="8">
@@ -679,12 +679,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>INE090A01021</t>
+          <t>INE062A01020</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ICICI Bank Ltd.</t>
+          <t>State Bank of India</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -698,34 +698,34 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>13811361</v>
+        <v>18844802</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>1387.5</v>
+        <v>1045.4</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>1916.3263</v>
+        <v>1970.0356</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1387.5</v>
+        <v>1045.4</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>1916.3263</v>
+        <v>1970.0356</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1373.6</v>
+        <v>1034.6</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>1897.1285</v>
+        <v>1949.6832</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>1.0119</v>
+        <v>1.0439</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>0.02309</v>
+        <v>0.02449</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>2.2818</v>
+        <v>2.3457</v>
       </c>
     </row>
     <row r="9">
@@ -734,12 +734,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>INE237A01036</t>
+          <t>INE090A01021</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Bank Ltd.</t>
+          <t>ICICI Bank Ltd.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -753,34 +753,34 @@
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>44549651</v>
+        <v>13616083</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>409</v>
+        <v>1387.5</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>1822.0807</v>
+        <v>1889.2315</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>409</v>
+        <v>1387.5</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>1822.0807</v>
+        <v>1889.2315</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>405.95</v>
+        <v>1373.6</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>1808.4931</v>
+        <v>1870.3052</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>0.7513</v>
+        <v>1.0119</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>0.0163</v>
+        <v>0.02276</v>
       </c>
       <c r="O9" s="9" t="n">
-        <v>2.1696</v>
+        <v>2.2495</v>
       </c>
     </row>
     <row r="10">
@@ -789,12 +789,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>INE040A01034</t>
+          <t>INE237A01036</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>HDFC Bank Ltd.</t>
+          <t>Kotak Mahindra Bank Ltd.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -808,34 +808,34 @@
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>18147664</v>
+        <v>45913877</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>796.3</v>
+        <v>409</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>1445.0985</v>
+        <v>1877.8776</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>796.3</v>
+        <v>409</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>1445.0985</v>
+        <v>1877.8776</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>793.2</v>
+        <v>405.95</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>1439.4727</v>
+        <v>1863.8738</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>0.3908</v>
+        <v>0.7513</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>0.00672</v>
+        <v>0.0168</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>1.7207</v>
+        <v>2.236</v>
       </c>
     </row>
     <row r="11">
@@ -844,12 +844,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>INE062A01020</t>
+          <t>INE040A01034</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>State Bank of India</t>
+          <t>HDFC Bank Ltd.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -863,34 +863,34 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>12921876</v>
+        <v>22368924</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>1045.4</v>
+        <v>796.3</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>1350.8529</v>
+        <v>1781.2374</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>1045.4</v>
+        <v>796.3</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>1350.8529</v>
+        <v>1781.2374</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1034.6</v>
+        <v>793.2</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>1336.8973</v>
+        <v>1774.3031</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>1.0439</v>
+        <v>0.3908</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>0.01679</v>
+        <v>0.00829</v>
       </c>
       <c r="O11" s="9" t="n">
-        <v>1.6085</v>
+        <v>2.1209</v>
       </c>
     </row>
     <row r="12">
@@ -908,14 +908,14 @@
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
       <c r="J12" s="13" t="n">
-        <v>6534.358</v>
+        <v>7518.382</v>
       </c>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="14" t="n">
-        <v>7.78</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -943,34 +943,34 @@
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>46412664</v>
+        <v>35197896</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>507.65</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>2356.1389</v>
+        <v>1786.8212</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>507.65</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>2356.1389</v>
+        <v>1786.8212</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>506.7</v>
       </c>
       <c r="L13" s="8" t="n">
-        <v>2351.7297</v>
+        <v>1783.4774</v>
       </c>
       <c r="M13" s="9" t="n">
         <v>0.1875</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>0.00526</v>
+        <v>0.00399</v>
       </c>
       <c r="O13" s="9" t="n">
-        <v>2.8055</v>
+        <v>2.1276</v>
       </c>
     </row>
     <row r="14">
@@ -998,34 +998,34 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>236418</v>
+        <v>1578988</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>1328.8</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>31.4152</v>
+        <v>209.8159</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>1328.8</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>31.4152</v>
+        <v>209.8159</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>1336.5</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>31.5973</v>
+        <v>211.0317</v>
       </c>
       <c r="M14" s="9" t="n">
         <v>-0.5760999999999999</v>
       </c>
       <c r="N14" s="10" t="n">
-        <v>-0.00022</v>
+        <v>-0.00144</v>
       </c>
       <c r="O14" s="9" t="n">
-        <v>0.0374</v>
+        <v>0.2498</v>
       </c>
     </row>
     <row r="15">
@@ -1043,14 +1043,14 @@
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
       <c r="J15" s="13" t="n">
-        <v>2387.554</v>
+        <v>1996.637</v>
       </c>
       <c r="K15" s="11" t="n"/>
       <c r="L15" s="11" t="n"/>
       <c r="M15" s="11" t="n"/>
       <c r="N15" s="11" t="n"/>
       <c r="O15" s="14" t="n">
-        <v>2.84</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="16">
@@ -1158,34 +1158,34 @@
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>1730467</v>
+        <v>1162731</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>17428</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>3015.8579</v>
+        <v>2026.4076</v>
       </c>
       <c r="I18" s="7" t="n">
         <v>17428</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>3015.8579</v>
+        <v>2026.4076</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>17864</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>3091.3062</v>
+        <v>2077.1027</v>
       </c>
       <c r="M18" s="9" t="n">
         <v>-2.4407</v>
       </c>
       <c r="N18" s="10" t="n">
-        <v>-0.08765000000000001</v>
+        <v>-0.05889</v>
       </c>
       <c r="O18" s="9" t="n">
-        <v>3.591</v>
+        <v>2.4129</v>
       </c>
     </row>
     <row r="19">
@@ -1203,14 +1203,14 @@
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
       <c r="J19" s="13" t="n">
-        <v>3015.858</v>
+        <v>2026.408</v>
       </c>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="14" t="n">
-        <v>3.59</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="20">
@@ -1238,34 +1238,34 @@
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>447043</v>
+        <v>1800259</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>4216.4</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>188.4912</v>
+        <v>759.0612</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>4216.4</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>188.4912</v>
+        <v>759.0612</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>4181.7</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>186.94</v>
+        <v>752.8143</v>
       </c>
       <c r="M20" s="9" t="n">
         <v>0.8298</v>
       </c>
       <c r="N20" s="10" t="n">
-        <v>0.00186</v>
+        <v>0.0075</v>
       </c>
       <c r="O20" s="9" t="n">
-        <v>0.2244</v>
+        <v>0.9038</v>
       </c>
     </row>
     <row r="21">
@@ -1283,14 +1283,14 @@
       <c r="H21" s="11" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="13" t="n">
-        <v>188.491</v>
+        <v>759.061</v>
       </c>
       <c r="K21" s="11" t="n"/>
       <c r="L21" s="11" t="n"/>
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
       <c r="O21" s="14" t="n">
-        <v>0.22</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="22">
@@ -1318,34 +1318,34 @@
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>61329599</v>
+        <v>62909282</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>435.4</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>2670.2907</v>
+        <v>2739.0701</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>435.4</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>2670.2907</v>
+        <v>2739.0701</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>441.75</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>2709.235</v>
+        <v>2779.0175</v>
       </c>
       <c r="M22" s="9" t="n">
         <v>-1.4375</v>
       </c>
       <c r="N22" s="10" t="n">
-        <v>-0.04571</v>
+        <v>-0.04688</v>
       </c>
       <c r="O22" s="9" t="n">
-        <v>3.1795</v>
+        <v>3.2614</v>
       </c>
     </row>
     <row r="23">
@@ -1363,14 +1363,14 @@
       <c r="H23" s="11" t="n"/>
       <c r="I23" s="11" t="n"/>
       <c r="J23" s="13" t="n">
-        <v>2670.291</v>
+        <v>2739.07</v>
       </c>
       <c r="K23" s="11" t="n"/>
       <c r="L23" s="11" t="n"/>
       <c r="M23" s="11" t="n"/>
       <c r="N23" s="11" t="n"/>
       <c r="O23" s="14" t="n">
-        <v>3.18</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="24">
@@ -1398,34 +1398,34 @@
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>11638773</v>
+        <v>8148052</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>2645.2</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>3078.6882</v>
+        <v>2155.3227</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>2645.2</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>3078.6882</v>
+        <v>2155.3227</v>
       </c>
       <c r="K24" s="7" t="n">
         <v>2667.5</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>3104.6427</v>
+        <v>2173.4929</v>
       </c>
       <c r="M24" s="9" t="n">
         <v>-0.836</v>
       </c>
       <c r="N24" s="10" t="n">
-        <v>-0.03065</v>
+        <v>-0.02146</v>
       </c>
       <c r="O24" s="9" t="n">
-        <v>3.6658</v>
+        <v>2.5664</v>
       </c>
     </row>
     <row r="25">
@@ -1443,14 +1443,14 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
       <c r="J25" s="13" t="n">
-        <v>3078.688</v>
+        <v>2155.323</v>
       </c>
       <c r="K25" s="11" t="n"/>
       <c r="L25" s="11" t="n"/>
       <c r="M25" s="11" t="n"/>
       <c r="N25" s="11" t="n"/>
       <c r="O25" s="14" t="n">
-        <v>3.67</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="26">
@@ -1478,34 +1478,34 @@
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>56330677</v>
+        <v>57027144</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>290</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>1633.5896</v>
+        <v>1653.7872</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>290</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>1633.5896</v>
+        <v>1653.7872</v>
       </c>
       <c r="K26" s="7" t="n">
         <v>290.35</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>1635.5612</v>
+        <v>1655.7831</v>
       </c>
       <c r="M26" s="9" t="n">
         <v>-0.1205</v>
       </c>
       <c r="N26" s="10" t="n">
-        <v>-0.00234</v>
+        <v>-0.00237</v>
       </c>
       <c r="O26" s="9" t="n">
-        <v>1.9451</v>
+        <v>1.9692</v>
       </c>
     </row>
     <row r="27">
@@ -1523,14 +1523,14 @@
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n"/>
       <c r="J27" s="13" t="n">
-        <v>1633.59</v>
+        <v>1653.787</v>
       </c>
       <c r="K27" s="11" t="n"/>
       <c r="L27" s="11" t="n"/>
       <c r="M27" s="11" t="n"/>
       <c r="N27" s="11" t="n"/>
       <c r="O27" s="14" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="28">
@@ -1558,34 +1558,34 @@
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>16308024</v>
+        <v>17672084</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>1059.5</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>1727.8351</v>
+        <v>1872.3573</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>1059.5</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>1727.8351</v>
+        <v>1872.3573</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>1089.7</v>
       </c>
       <c r="L28" s="8" t="n">
-        <v>1777.0854</v>
+        <v>1925.727</v>
       </c>
       <c r="M28" s="9" t="n">
         <v>-2.7714</v>
       </c>
       <c r="N28" s="10" t="n">
-        <v>-0.05702</v>
+        <v>-0.06179</v>
       </c>
       <c r="O28" s="9" t="n">
-        <v>2.0574</v>
+        <v>2.2294</v>
       </c>
     </row>
     <row r="29">
@@ -1603,14 +1603,14 @@
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n"/>
       <c r="J29" s="13" t="n">
-        <v>1727.835</v>
+        <v>1872.357</v>
       </c>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="11" t="n"/>
       <c r="M29" s="11" t="n"/>
       <c r="N29" s="11" t="n"/>
       <c r="O29" s="14" t="n">
-        <v>2.06</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="30">
@@ -1638,34 +1638,34 @@
         </is>
       </c>
       <c r="F30" s="6" t="n">
-        <v>10071632</v>
+        <v>8691151</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>3025.6</v>
       </c>
       <c r="H30" s="8" t="n">
-        <v>3047.273</v>
+        <v>2629.5946</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>3025.6</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>3047.273</v>
+        <v>2629.5946</v>
       </c>
       <c r="K30" s="7" t="n">
         <v>3129.9</v>
       </c>
       <c r="L30" s="8" t="n">
-        <v>3152.3201</v>
+        <v>2720.2434</v>
       </c>
       <c r="M30" s="9" t="n">
         <v>-3.3324</v>
       </c>
       <c r="N30" s="10" t="n">
-        <v>-0.12091</v>
+        <v>-0.10434</v>
       </c>
       <c r="O30" s="9" t="n">
-        <v>3.6284</v>
+        <v>3.1311</v>
       </c>
     </row>
     <row r="31">
@@ -1693,34 +1693,34 @@
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>18905507</v>
+        <v>16367225</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>980.4</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>1853.4959</v>
+        <v>1604.6427</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>980.4</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>1853.4959</v>
+        <v>1604.6427</v>
       </c>
       <c r="K31" s="7" t="n">
         <v>990.95</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>1873.4412</v>
+        <v>1621.9102</v>
       </c>
       <c r="M31" s="9" t="n">
         <v>-1.0646</v>
       </c>
       <c r="N31" s="10" t="n">
-        <v>-0.0235</v>
+        <v>-0.02034</v>
       </c>
       <c r="O31" s="9" t="n">
-        <v>2.207</v>
+        <v>1.9107</v>
       </c>
     </row>
     <row r="32">
@@ -1738,14 +1738,14 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="13" t="n">
-        <v>4900.769</v>
+        <v>4234.237</v>
       </c>
       <c r="K32" s="11" t="n"/>
       <c r="L32" s="11" t="n"/>
       <c r="M32" s="11" t="n"/>
       <c r="N32" s="11" t="n"/>
       <c r="O32" s="14" t="n">
-        <v>5.83</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="33">
@@ -1773,34 +1773,34 @@
         </is>
       </c>
       <c r="F33" s="6" t="n">
-        <v>8110031</v>
+        <v>8143041</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>1123.35</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>911.0403</v>
+        <v>914.7485</v>
       </c>
       <c r="I33" s="7" t="n">
         <v>1123.35</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>911.0403</v>
+        <v>914.7485</v>
       </c>
       <c r="K33" s="7" t="n">
         <v>1081.7</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>877.2621</v>
+        <v>880.8327</v>
       </c>
       <c r="M33" s="9" t="n">
         <v>3.8504</v>
       </c>
       <c r="N33" s="10" t="n">
-        <v>0.04177</v>
+        <v>0.04194</v>
       </c>
       <c r="O33" s="9" t="n">
-        <v>1.0848</v>
+        <v>1.0892</v>
       </c>
     </row>
     <row r="34">
@@ -1818,14 +1818,14 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="11" t="n"/>
       <c r="J34" s="13" t="n">
-        <v>911.04</v>
+        <v>914.749</v>
       </c>
       <c r="K34" s="11" t="n"/>
       <c r="L34" s="11" t="n"/>
       <c r="M34" s="11" t="n"/>
       <c r="N34" s="11" t="n"/>
       <c r="O34" s="14" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="35">
@@ -1853,34 +1853,34 @@
         </is>
       </c>
       <c r="F35" s="6" t="n">
-        <v>11398072</v>
+        <v>10004912</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>2094.7</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>2387.5541</v>
+        <v>2095.7289</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>2094.7</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>2387.5541</v>
+        <v>2095.7289</v>
       </c>
       <c r="K35" s="7" t="n">
         <v>2109</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>2403.8534</v>
+        <v>2110.0359</v>
       </c>
       <c r="M35" s="9" t="n">
         <v>-0.678</v>
       </c>
       <c r="N35" s="10" t="n">
-        <v>-0.01927</v>
+        <v>-0.01692</v>
       </c>
       <c r="O35" s="9" t="n">
-        <v>2.8429</v>
+        <v>2.4954</v>
       </c>
     </row>
     <row r="36">
@@ -1908,34 +1908,34 @@
         </is>
       </c>
       <c r="F36" s="6" t="n">
-        <v>17499815</v>
+        <v>18091051</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>1041.2</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>1822.0807</v>
+        <v>1883.6402</v>
       </c>
       <c r="I36" s="7" t="n">
         <v>1041.2</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>1822.0807</v>
+        <v>1883.6402</v>
       </c>
       <c r="K36" s="7" t="n">
         <v>1056.6</v>
       </c>
       <c r="L36" s="8" t="n">
-        <v>1849.0305</v>
+        <v>1911.5004</v>
       </c>
       <c r="M36" s="9" t="n">
         <v>-1.4575</v>
       </c>
       <c r="N36" s="10" t="n">
-        <v>-0.03162</v>
+        <v>-0.03269</v>
       </c>
       <c r="O36" s="9" t="n">
-        <v>2.1696</v>
+        <v>2.2429</v>
       </c>
     </row>
     <row r="37">
@@ -1953,14 +1953,14 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="11" t="n"/>
       <c r="J37" s="13" t="n">
-        <v>4209.635</v>
+        <v>3979.369</v>
       </c>
       <c r="K37" s="11" t="n"/>
       <c r="L37" s="11" t="n"/>
       <c r="M37" s="11" t="n"/>
       <c r="N37" s="11" t="n"/>
       <c r="O37" s="14" t="n">
-        <v>5.01</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="38">
@@ -2203,34 +2203,34 @@
         </is>
       </c>
       <c r="F43" s="6" t="n">
-        <v>24718201</v>
+        <v>28217630</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>953.2</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>2356.1389</v>
+        <v>2689.7045</v>
       </c>
       <c r="I43" s="7" t="n">
         <v>953.2</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>2356.1389</v>
+        <v>2689.7045</v>
       </c>
       <c r="K43" s="7" t="n">
         <v>976.6</v>
       </c>
       <c r="L43" s="8" t="n">
-        <v>2413.9795</v>
+        <v>2755.7337</v>
       </c>
       <c r="M43" s="9" t="n">
         <v>-2.3961</v>
       </c>
       <c r="N43" s="10" t="n">
-        <v>-0.06722</v>
+        <v>-0.07674</v>
       </c>
       <c r="O43" s="9" t="n">
-        <v>2.8055</v>
+        <v>3.2027</v>
       </c>
     </row>
     <row r="44">
@@ -2248,14 +2248,14 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="11" t="n"/>
       <c r="J44" s="13" t="n">
-        <v>2356.139</v>
+        <v>2689.704</v>
       </c>
       <c r="K44" s="11" t="n"/>
       <c r="L44" s="11" t="n"/>
       <c r="M44" s="11" t="n"/>
       <c r="N44" s="11" t="n"/>
       <c r="O44" s="14" t="n">
-        <v>2.81</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="45">
@@ -2363,34 +2363,34 @@
         </is>
       </c>
       <c r="F47" s="6" t="n">
-        <v>11678508</v>
+        <v>13456130</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>1318.1</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>1539.3441</v>
+        <v>1773.6525</v>
       </c>
       <c r="I47" s="7" t="n">
         <v>1318.1</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>1539.3441</v>
+        <v>1773.6525</v>
       </c>
       <c r="K47" s="7" t="n">
         <v>1313.6</v>
       </c>
       <c r="L47" s="8" t="n">
-        <v>1534.0888</v>
+        <v>1767.5972</v>
       </c>
       <c r="M47" s="9" t="n">
         <v>0.3426</v>
       </c>
       <c r="N47" s="10" t="n">
-        <v>0.00628</v>
+        <v>0.00724</v>
       </c>
       <c r="O47" s="9" t="n">
-        <v>1.8329</v>
+        <v>2.1119</v>
       </c>
     </row>
     <row r="48">
@@ -2408,14 +2408,14 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="11" t="n"/>
       <c r="J48" s="13" t="n">
-        <v>1539.344</v>
+        <v>1773.652</v>
       </c>
       <c r="K48" s="11" t="n"/>
       <c r="L48" s="11" t="n"/>
       <c r="M48" s="11" t="n"/>
       <c r="N48" s="11" t="n"/>
       <c r="O48" s="14" t="n">
-        <v>1.83</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="49">
@@ -2443,34 +2443,34 @@
         </is>
       </c>
       <c r="F49" s="6" t="n">
-        <v>1310233</v>
+        <v>1338681</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>6713.5</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>879.6249</v>
+        <v>898.7234999999999</v>
       </c>
       <c r="I49" s="7" t="n">
         <v>6713.5</v>
       </c>
       <c r="J49" s="8" t="n">
-        <v>879.6249</v>
+        <v>898.7234999999999</v>
       </c>
       <c r="K49" s="7" t="n">
         <v>6753.5</v>
       </c>
       <c r="L49" s="8" t="n">
-        <v>884.8659</v>
+        <v>904.0782</v>
       </c>
       <c r="M49" s="9" t="n">
         <v>-0.5923</v>
       </c>
       <c r="N49" s="10" t="n">
-        <v>-0.0062</v>
+        <v>-0.00634</v>
       </c>
       <c r="O49" s="9" t="n">
-        <v>1.0474</v>
+        <v>1.0701</v>
       </c>
     </row>
     <row r="50">
@@ -2488,14 +2488,14 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="11" t="n"/>
       <c r="J50" s="13" t="n">
-        <v>879.625</v>
+        <v>898.723</v>
       </c>
       <c r="K50" s="11" t="n"/>
       <c r="L50" s="11" t="n"/>
       <c r="M50" s="11" t="n"/>
       <c r="N50" s="11" t="n"/>
       <c r="O50" s="14" t="n">
-        <v>1.05</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="51">
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F51" s="6" t="n">
-        <v>58002756</v>
+        <v>66828928</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>352.05</v>
       </c>
       <c r="H51" s="8" t="n">
-        <v>2041.987</v>
+        <v>2352.7124</v>
       </c>
       <c r="I51" s="7" t="n">
         <v>352.05</v>
       </c>
       <c r="J51" s="8" t="n">
-        <v>2041.987</v>
+        <v>2352.7124</v>
       </c>
       <c r="K51" s="7" t="n">
         <v>357.05</v>
       </c>
       <c r="L51" s="8" t="n">
-        <v>2070.9884</v>
+        <v>2386.1269</v>
       </c>
       <c r="M51" s="9" t="n">
         <v>-1.4004</v>
       </c>
       <c r="N51" s="10" t="n">
-        <v>-0.03405</v>
+        <v>-0.03923</v>
       </c>
       <c r="O51" s="9" t="n">
-        <v>2.4314</v>
+        <v>2.8014</v>
       </c>
     </row>
     <row r="52">
@@ -2578,34 +2578,34 @@
         </is>
       </c>
       <c r="F52" s="6" t="n">
-        <v>49328158</v>
+        <v>50731155</v>
       </c>
       <c r="G52" s="7" t="n">
         <v>229.27</v>
       </c>
       <c r="H52" s="8" t="n">
-        <v>1130.9467</v>
+        <v>1163.1132</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>229.27</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>1130.9467</v>
+        <v>1163.1132</v>
       </c>
       <c r="K52" s="7" t="n">
         <v>229.76</v>
       </c>
       <c r="L52" s="8" t="n">
-        <v>1133.3638</v>
+        <v>1165.599</v>
       </c>
       <c r="M52" s="9" t="n">
         <v>-0.2133</v>
       </c>
       <c r="N52" s="10" t="n">
-        <v>-0.00287</v>
+        <v>-0.00295</v>
       </c>
       <c r="O52" s="9" t="n">
-        <v>1.3466</v>
+        <v>1.3849</v>
       </c>
     </row>
     <row r="53">
@@ -2633,34 +2633,34 @@
         </is>
       </c>
       <c r="F53" s="6" t="n">
-        <v>4167023</v>
+        <v>5401997</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>1507.8</v>
       </c>
       <c r="H53" s="8" t="n">
-        <v>628.3037</v>
+        <v>814.5131</v>
       </c>
       <c r="I53" s="7" t="n">
         <v>1507.8</v>
       </c>
       <c r="J53" s="8" t="n">
-        <v>628.3037</v>
+        <v>814.5131</v>
       </c>
       <c r="K53" s="7" t="n">
         <v>1495.9</v>
       </c>
       <c r="L53" s="8" t="n">
-        <v>623.345</v>
+        <v>808.0847</v>
       </c>
       <c r="M53" s="9" t="n">
         <v>0.7955</v>
       </c>
       <c r="N53" s="10" t="n">
-        <v>0.00595</v>
+        <v>0.00771</v>
       </c>
       <c r="O53" s="9" t="n">
-        <v>0.7481</v>
+        <v>0.9698</v>
       </c>
     </row>
     <row r="54">
@@ -2688,34 +2688,34 @@
         </is>
       </c>
       <c r="F54" s="6" t="n">
-        <v>1095560</v>
+        <v>11443887</v>
       </c>
       <c r="G54" s="7" t="n">
         <v>573.5</v>
       </c>
       <c r="H54" s="8" t="n">
-        <v>62.8304</v>
+        <v>656.3069</v>
       </c>
       <c r="I54" s="7" t="n">
         <v>573.5</v>
       </c>
       <c r="J54" s="8" t="n">
-        <v>62.8304</v>
+        <v>656.3069</v>
       </c>
       <c r="K54" s="7" t="n">
         <v>574.4</v>
       </c>
       <c r="L54" s="8" t="n">
-        <v>62.929</v>
+        <v>657.3369</v>
       </c>
       <c r="M54" s="9" t="n">
         <v>-0.1567</v>
       </c>
       <c r="N54" s="10" t="n">
-        <v>-0.00012</v>
+        <v>-0.00122</v>
       </c>
       <c r="O54" s="9" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.7815</v>
       </c>
     </row>
     <row r="55">
@@ -2733,14 +2733,14 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="11" t="n"/>
       <c r="J55" s="13" t="n">
-        <v>3864.068</v>
+        <v>4986.646</v>
       </c>
       <c r="K55" s="11" t="n"/>
       <c r="L55" s="11" t="n"/>
       <c r="M55" s="11" t="n"/>
       <c r="N55" s="11" t="n"/>
       <c r="O55" s="14" t="n">
-        <v>4.6</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="56">
@@ -2768,34 +2768,34 @@
         </is>
       </c>
       <c r="F56" s="6" t="n">
-        <v>25785378</v>
+        <v>24807807</v>
       </c>
       <c r="G56" s="7" t="n">
         <v>621.35</v>
       </c>
       <c r="H56" s="8" t="n">
-        <v>1602.1745</v>
+        <v>1541.4331</v>
       </c>
       <c r="I56" s="7" t="n">
         <v>621.35</v>
       </c>
       <c r="J56" s="8" t="n">
-        <v>1602.1745</v>
+        <v>1541.4331</v>
       </c>
       <c r="K56" s="7" t="n">
         <v>618.15</v>
       </c>
       <c r="L56" s="8" t="n">
-        <v>1593.9231</v>
+        <v>1533.4946</v>
       </c>
       <c r="M56" s="9" t="n">
         <v>0.5177</v>
       </c>
       <c r="N56" s="10" t="n">
-        <v>0.00988</v>
+        <v>0.0095</v>
       </c>
       <c r="O56" s="9" t="n">
-        <v>1.9077</v>
+        <v>1.8354</v>
       </c>
     </row>
     <row r="57">
@@ -2868,14 +2868,14 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="11" t="n"/>
       <c r="J58" s="13" t="n">
-        <v>2683.429</v>
+        <v>2622.688</v>
       </c>
       <c r="K58" s="11" t="n"/>
       <c r="L58" s="11" t="n"/>
       <c r="M58" s="11" t="n"/>
       <c r="N58" s="11" t="n"/>
       <c r="O58" s="14" t="n">
-        <v>3.19</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="59">
@@ -2884,12 +2884,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>INE956O01016</t>
+          <t>INE0VDM01015</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Lenskart Solutions Ltd.</t>
+          <t>Meesho Ltd.</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -2899,38 +2899,38 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>tactical</t>
+          <t>structural</t>
         </is>
       </c>
       <c r="F59" s="6" t="n">
-        <v>60496918</v>
+        <v>157572215</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>508.9</v>
+        <v>186.45</v>
       </c>
       <c r="H59" s="8" t="n">
-        <v>3078.6882</v>
+        <v>2937.9339</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>508.9</v>
+        <v>186.45</v>
       </c>
       <c r="J59" s="8" t="n">
-        <v>3078.6882</v>
+        <v>2937.9339</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>516.35</v>
+        <v>188.37</v>
       </c>
       <c r="L59" s="8" t="n">
-        <v>3123.7584</v>
+        <v>2968.1878</v>
       </c>
       <c r="M59" s="9" t="n">
-        <v>-1.4428</v>
+        <v>-1.0193</v>
       </c>
       <c r="N59" s="10" t="n">
-        <v>-0.05289</v>
+        <v>-0.03566</v>
       </c>
       <c r="O59" s="9" t="n">
-        <v>3.6658</v>
+        <v>3.4982</v>
       </c>
     </row>
     <row r="60">
@@ -2939,12 +2939,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>INE192R01011</t>
+          <t>INE956O01016</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Avenue Supermarts Ltd.</t>
+          <t>Lenskart Solutions Ltd.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2954,38 +2954,38 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>structural</t>
+          <t>tactical</t>
         </is>
       </c>
       <c r="F60" s="6" t="n">
-        <v>4754778</v>
+        <v>42694550</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>4294.6</v>
+        <v>508.9</v>
       </c>
       <c r="H60" s="8" t="n">
-        <v>2041.987</v>
+        <v>2172.7256</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>4294.6</v>
+        <v>508.9</v>
       </c>
       <c r="J60" s="8" t="n">
-        <v>2041.987</v>
+        <v>2172.7256</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>4336</v>
+        <v>516.35</v>
       </c>
       <c r="L60" s="8" t="n">
-        <v>2061.6717</v>
+        <v>2204.5331</v>
       </c>
       <c r="M60" s="9" t="n">
-        <v>-0.9548</v>
+        <v>-1.4428</v>
       </c>
       <c r="N60" s="10" t="n">
-        <v>-0.02322</v>
+        <v>-0.03733</v>
       </c>
       <c r="O60" s="9" t="n">
-        <v>2.4314</v>
+        <v>2.5871</v>
       </c>
     </row>
     <row r="61">
@@ -2994,12 +2994,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>INE01EA01019</t>
+          <t>INE192R01011</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Vishal Mega Mart Ltd.</t>
+          <t>Avenue Supermarts Ltd.</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -3013,34 +3013,34 @@
         </is>
       </c>
       <c r="F61" s="6" t="n">
-        <v>153850465</v>
+        <v>3619667</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>116.39</v>
+        <v>4294.6</v>
       </c>
       <c r="H61" s="8" t="n">
-        <v>1790.6656</v>
+        <v>1554.5022</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>116.39</v>
+        <v>4294.6</v>
       </c>
       <c r="J61" s="8" t="n">
-        <v>1790.6656</v>
+        <v>1554.5022</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>118.97</v>
+        <v>4336</v>
       </c>
       <c r="L61" s="8" t="n">
-        <v>1830.359</v>
+        <v>1569.4876</v>
       </c>
       <c r="M61" s="9" t="n">
-        <v>-2.1686</v>
+        <v>-0.9548</v>
       </c>
       <c r="N61" s="10" t="n">
-        <v>-0.04624</v>
+        <v>-0.01767</v>
       </c>
       <c r="O61" s="9" t="n">
-        <v>2.1322</v>
+        <v>1.851</v>
       </c>
     </row>
     <row r="62">
@@ -3049,12 +3049,12 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>INE0VDM01015</t>
+          <t>INE01EA01019</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Meesho Ltd.</t>
+          <t>Vishal Mega Mart Ltd.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -3068,34 +3068,34 @@
         </is>
       </c>
       <c r="F62" s="6" t="n">
-        <v>87615427</v>
+        <v>126546423</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>186.45</v>
+        <v>116.39</v>
       </c>
       <c r="H62" s="8" t="n">
-        <v>1633.5896</v>
+        <v>1472.8738</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>186.45</v>
+        <v>116.39</v>
       </c>
       <c r="J62" s="8" t="n">
-        <v>1633.5896</v>
+        <v>1472.8738</v>
       </c>
       <c r="K62" s="7" t="n">
-        <v>188.37</v>
+        <v>118.97</v>
       </c>
       <c r="L62" s="8" t="n">
-        <v>1650.4118</v>
+        <v>1505.5228</v>
       </c>
       <c r="M62" s="9" t="n">
-        <v>-1.0193</v>
+        <v>-2.1686</v>
       </c>
       <c r="N62" s="10" t="n">
-        <v>-0.01983</v>
+        <v>-0.03803</v>
       </c>
       <c r="O62" s="9" t="n">
-        <v>1.9451</v>
+        <v>1.7538</v>
       </c>
     </row>
     <row r="63">
@@ -3123,34 +3123,34 @@
         </is>
       </c>
       <c r="F63" s="6" t="n">
-        <v>48280866</v>
+        <v>33998196</v>
       </c>
       <c r="G63" s="7" t="n">
         <v>240.75</v>
       </c>
       <c r="H63" s="8" t="n">
-        <v>1162.3618</v>
+        <v>818.5066</v>
       </c>
       <c r="I63" s="7" t="n">
         <v>240.75</v>
       </c>
       <c r="J63" s="8" t="n">
-        <v>1162.3618</v>
+        <v>818.5066</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>244.2</v>
       </c>
       <c r="L63" s="8" t="n">
-        <v>1179.0187</v>
+        <v>830.2359</v>
       </c>
       <c r="M63" s="9" t="n">
         <v>-1.4128</v>
       </c>
       <c r="N63" s="10" t="n">
-        <v>-0.01955</v>
+        <v>-0.01377</v>
       </c>
       <c r="O63" s="9" t="n">
-        <v>1.384</v>
+        <v>0.9746</v>
       </c>
     </row>
     <row r="64">
@@ -3278,14 +3278,14 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="11" t="n"/>
       <c r="J66" s="13" t="n">
-        <v>10384.057</v>
+        <v>9633.307000000001</v>
       </c>
       <c r="K66" s="11" t="n"/>
       <c r="L66" s="11" t="n"/>
       <c r="M66" s="11" t="n"/>
       <c r="N66" s="11" t="n"/>
       <c r="O66" s="14" t="n">
-        <v>12.36</v>
+        <v>11.47</v>
       </c>
     </row>
     <row r="67">
@@ -3313,34 +3313,34 @@
         </is>
       </c>
       <c r="F67" s="6" t="n">
-        <v>10184855</v>
+        <v>8342609</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>1850.7</v>
       </c>
       <c r="H67" s="8" t="n">
-        <v>1884.9111</v>
+        <v>1543.9666</v>
       </c>
       <c r="I67" s="7" t="n">
         <v>1850.7</v>
       </c>
       <c r="J67" s="8" t="n">
-        <v>1884.9111</v>
+        <v>1543.9666</v>
       </c>
       <c r="K67" s="7" t="n">
         <v>1877.3</v>
       </c>
       <c r="L67" s="8" t="n">
-        <v>1912.0028</v>
+        <v>1566.158</v>
       </c>
       <c r="M67" s="9" t="n">
         <v>-1.4169</v>
       </c>
       <c r="N67" s="10" t="n">
-        <v>-0.0318</v>
+        <v>-0.02605</v>
       </c>
       <c r="O67" s="9" t="n">
-        <v>2.2444</v>
+        <v>1.8384</v>
       </c>
     </row>
     <row r="68">
@@ -3358,14 +3358,14 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="11" t="n"/>
       <c r="J68" s="13" t="n">
-        <v>1884.911</v>
+        <v>1543.967</v>
       </c>
       <c r="K68" s="11" t="n"/>
       <c r="L68" s="11" t="n"/>
       <c r="M68" s="11" t="n"/>
       <c r="N68" s="11" t="n"/>
       <c r="O68" s="14" t="n">
-        <v>2.24</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="69">
@@ -3473,34 +3473,34 @@
         </is>
       </c>
       <c r="F71" s="6" t="n">
-        <v>1152851</v>
+        <v>1260724</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>5450</v>
       </c>
       <c r="H71" s="8" t="n">
-        <v>628.3038</v>
+        <v>687.0946</v>
       </c>
       <c r="I71" s="7" t="n">
         <v>5450</v>
       </c>
       <c r="J71" s="8" t="n">
-        <v>628.3038</v>
+        <v>687.0946</v>
       </c>
       <c r="K71" s="7" t="n">
         <v>5207.2</v>
       </c>
       <c r="L71" s="8" t="n">
-        <v>600.3126</v>
+        <v>656.4842</v>
       </c>
       <c r="M71" s="9" t="n">
         <v>4.6628</v>
       </c>
       <c r="N71" s="10" t="n">
-        <v>0.03488</v>
+        <v>0.03815</v>
       </c>
       <c r="O71" s="9" t="n">
-        <v>0.7481</v>
+        <v>0.8181</v>
       </c>
     </row>
     <row r="72">
@@ -3518,14 +3518,14 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="11" t="n"/>
       <c r="J72" s="13" t="n">
-        <v>628.304</v>
+        <v>687.095</v>
       </c>
       <c r="K72" s="11" t="n"/>
       <c r="L72" s="11" t="n"/>
       <c r="M72" s="11" t="n"/>
       <c r="N72" s="11" t="n"/>
       <c r="O72" s="14" t="n">
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="74">
@@ -3535,7 +3535,7 @@
         </is>
       </c>
       <c r="C74" s="15" t="n">
-        <v>60888.043</v>
+        <v>60888.04</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3550,7 +3550,7 @@
         </is>
       </c>
       <c r="C75" s="15" t="n">
-        <v>23095.457</v>
+        <v>23095.46</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3595,7 +3595,7 @@
         </is>
       </c>
       <c r="C78" s="15" t="n">
-        <v>-0.6598000000000001</v>
+        <v>-0.5835</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>

</xml_diff>